<commit_message>
1952/53: opravit mistra dle PDF+web (M: Vítkovice → Spartak Praha Sokolovo)
PDF finálový turnaj: 1. Spartak Praha Sokolovo 9 b = mistr (před Vítkovicemi 6 b).
Ověřeno webem: první titul Sparty 1952/53 (hrající trenér Zábrodský). M badge byl
chybně u Baník VŽKG Vítkovice (vítěz základní skupiny, ne finále). M přesunut na
Spartak Praha Sokolovo ve finálovém bloku. META mistr=Spartak Praha Sokolovo.
</commit_message>
<xml_diff>
--- a/data/S1952_53_FINAL.xlsx
+++ b/data/S1952_53_FINAL.xlsx
@@ -1990,11 +1990,6 @@
           <t>Baník VŽKG Vítkovice</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
       <c r="F21" t="n">
         <v>12</v>
       </c>
@@ -2605,6 +2600,11 @@
       <c r="D29" t="inlineStr">
         <is>
           <t>Spartak Praha Sokolovo</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -24282,7 +24282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -24489,6 +24489,13 @@
       <c r="D15" t="inlineStr">
         <is>
           <t>TODO-auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mistrovství republiky 1952/53: základní skupiny → finálový turnaj. Mistr Spartak Praha Sokolovo (před Vítkovicemi). Doloženo PDF i webem.</t>
         </is>
       </c>
     </row>
@@ -24958,8 +24965,6 @@
           <t>NODE_S1952_53_0001</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25015,8 +25020,6 @@
           <t>NODE_S1952_53_0001</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25366,8 +25369,6 @@
           <t>NODE_S1952_53_0008</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25685,8 +25686,6 @@
           <t>NODE_S1952_53_0018</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26046,8 +26045,6 @@
           <t>NODE_S1952_53_0026</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26229,8 +26226,6 @@
           <t>NODE_S1952_53_0030</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26605,8 +26600,6 @@
           <t>NODE_S1952_53_0037</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27122,8 +27115,6 @@
           <t>NODE_S1952_53_0049</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -51443,7 +51434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51610,7 +51601,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bez L15 kvalifikace. Civilní krajští přeborníci nemohli postoupit; soutěž byla zúžena na 18 účastníků.</t>
+          <t>Mistr Spartak Praha Sokolovo — vítěz finálového turnaje (1., 9 b) před Vítkovicemi a Č. Budějovicemi (první titul Sparty, hrající trenér Zábrodský). M badge opraven (byl chybně u Baník VŽKG Vítkovice, vítěze základní skupiny). Pozn.: kluby přejmenovány od 12.12.1952 (DSO Baník/Slovan/Tatran…).</t>
         </is>
       </c>
     </row>
@@ -51851,6 +51842,18 @@
       <c r="B34" t="inlineStr">
         <is>
           <t>Žilinský</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>mistr</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>TJ Spartak Praha Sokolovo</t>
         </is>
       </c>
     </row>

</xml_diff>